<commit_message>
mod: actualizar tracker con protección de datos personales
</commit_message>
<xml_diff>
--- a/outputs/ldsm-identidad-20260729/Tracker_Implementacion_Identidad_y_Registro_Movil_LDSM.xlsx
+++ b/outputs/ldsm-identidad-20260729/Tracker_Implementacion_Identidad_y_Registro_Movil_LDSM.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Plan" sheetId="1" r:id="Rb2d490ceab4a48b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Plan" sheetId="1" r:id="R127d0521483c4fd9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1198,7 +1198,7 @@
       <x:c r="N6" s="44"/>
       <x:c r="O6" s="45" t="n">
         <x:f>COUNTIF($E$10:$E$39,"Completada")</x:f>
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="P6" s="46"/>
       <x:c r="Q6" s="46"/>
@@ -2796,24 +2796,25 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="E25" s="8" t="str">
-        <x:v>No iniciada</x:v>
+        <x:v>Completada</x:v>
       </x:c>
       <x:c r="F25" s="8" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="G25" s="49" t="n">
-        <x:v>46275</x:v>
+        <x:v>46235</x:v>
       </x:c>
       <x:c r="H25" s="49" t="n">
-        <x:v>46283</x:v>
+        <x:v>46235</x:v>
       </x:c>
       <x:c r="I25" s="11" t="n">
         <x:f t="shared" si="1">IF(OR(G25="",H25="",H25&lt;G25),"",H25-G25+1)</x:f>
-        <x:v>9</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J25" s="15"/>
-      <x:c r="K25" s="12" t="str">
+      <x:c r="K25" s="12" t="n">
         <x:f t="shared" si="4">IF(OR($G25="",$H25="",$H25&lt;$G25),"",IF(AND(K$9&lt;=$H25,K$9+6&gt;=$G25),1,""))</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L25" s="13" t="str">
         <x:f t="shared" si="4">IF(OR($G25="",$H25="",$H25&lt;$G25),"",IF(AND(L$9&lt;=$H25,L$9+6&gt;=$G25),1,""))</x:f>
@@ -2830,13 +2831,11 @@
       <x:c r="P25" s="13" t="str">
         <x:f t="shared" si="4">IF(OR($G25="",$H25="",$H25&lt;$G25),"",IF(AND(P$9&lt;=$H25,P$9+6&gt;=$G25),1,""))</x:f>
       </x:c>
-      <x:c r="Q25" s="12" t="n">
+      <x:c r="Q25" s="12" t="str">
         <x:f t="shared" si="4">IF(OR($G25="",$H25="",$H25&lt;$G25),"",IF(AND(Q$9&lt;=$H25,Q$9+6&gt;=$G25),1,""))</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="R25" s="13" t="n">
+      </x:c>
+      <x:c r="R25" s="13" t="str">
         <x:f t="shared" si="4">IF(OR($G25="",$H25="",$H25&lt;$G25),"",IF(AND(R$9&lt;=$H25,R$9+6&gt;=$G25),1,""))</x:f>
-        <x:v>1</x:v>
       </x:c>
       <x:c r="S25" s="12" t="str">
         <x:f t="shared" si="4">IF(OR($G25="",$H25="",$H25&lt;$G25),"",IF(AND(S$9&lt;=$H25,S$9+6&gt;=$G25),1,""))</x:f>

</xml_diff>

<commit_message>
mod: actualizar tracker con validadores por país
</commit_message>
<xml_diff>
--- a/outputs/ldsm-identidad-20260729/Tracker_Implementacion_Identidad_y_Registro_Movil_LDSM.xlsx
+++ b/outputs/ldsm-identidad-20260729/Tracker_Implementacion_Identidad_y_Registro_Movil_LDSM.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Plan" sheetId="1" r:id="R127d0521483c4fd9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Plan" sheetId="1" r:id="R59e793671e1a4ac2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1198,7 +1198,7 @@
       <x:c r="N6" s="44"/>
       <x:c r="O6" s="45" t="n">
         <x:f>COUNTIF($E$10:$E$39,"Completada")</x:f>
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="P6" s="46"/>
       <x:c r="Q6" s="46"/>
@@ -2974,24 +2974,25 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="E27" s="8" t="str">
-        <x:v>No iniciada</x:v>
+        <x:v>Completada</x:v>
       </x:c>
       <x:c r="F27" s="8" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="G27" s="49" t="n">
-        <x:v>46283</x:v>
+        <x:v>46235</x:v>
       </x:c>
       <x:c r="H27" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46235</x:v>
       </x:c>
       <x:c r="I27" s="11" t="n">
         <x:f t="shared" si="1">IF(OR(G27="",H27="",H27&lt;G27),"",H27-G27+1)</x:f>
-        <x:v>13</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J27" s="15"/>
-      <x:c r="K27" s="12" t="str">
+      <x:c r="K27" s="12" t="n">
         <x:f t="shared" si="4">IF(OR($G27="",$H27="",$H27&lt;$G27),"",IF(AND(K$9&lt;=$H27,K$9+6&gt;=$G27),1,""))</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L27" s="13" t="str">
         <x:f t="shared" si="4">IF(OR($G27="",$H27="",$H27&lt;$G27),"",IF(AND(L$9&lt;=$H27,L$9+6&gt;=$G27),1,""))</x:f>
@@ -3011,17 +3012,14 @@
       <x:c r="Q27" s="12" t="str">
         <x:f t="shared" si="4">IF(OR($G27="",$H27="",$H27&lt;$G27),"",IF(AND(Q$9&lt;=$H27,Q$9+6&gt;=$G27),1,""))</x:f>
       </x:c>
-      <x:c r="R27" s="13" t="n">
+      <x:c r="R27" s="13" t="str">
         <x:f t="shared" si="4">IF(OR($G27="",$H27="",$H27&lt;$G27),"",IF(AND(R$9&lt;=$H27,R$9+6&gt;=$G27),1,""))</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="S27" s="12" t="n">
+      </x:c>
+      <x:c r="S27" s="12" t="str">
         <x:f t="shared" si="4">IF(OR($G27="",$H27="",$H27&lt;$G27),"",IF(AND(S$9&lt;=$H27,S$9+6&gt;=$G27),1,""))</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="T27" s="13" t="n">
+      </x:c>
+      <x:c r="T27" s="13" t="str">
         <x:f t="shared" si="4">IF(OR($G27="",$H27="",$H27&lt;$G27),"",IF(AND(T$9&lt;=$H27,T$9+6&gt;=$G27),1,""))</x:f>
-        <x:v>1</x:v>
       </x:c>
       <x:c r="U27" s="12" t="str">
         <x:f t="shared" si="5">IF(OR($G27="",$H27="",$H27&lt;$G27),"",IF(AND(U$9&lt;=$H27,U$9+6&gt;=$G27),1,""))</x:f>

</xml_diff>

<commit_message>
mod: actualizar tracker con registro móvil
</commit_message>
<xml_diff>
--- a/outputs/ldsm-identidad-20260729/Tracker_Implementacion_Identidad_y_Registro_Movil_LDSM.xlsx
+++ b/outputs/ldsm-identidad-20260729/Tracker_Implementacion_Identidad_y_Registro_Movil_LDSM.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Plan" sheetId="1" r:id="R59e793671e1a4ac2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Plan" sheetId="1" r:id="Rd915ee891ba54079"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1198,7 +1198,7 @@
       <x:c r="N6" s="44"/>
       <x:c r="O6" s="45" t="n">
         <x:f>COUNTIF($E$10:$E$39,"Completada")</x:f>
-        <x:v>19</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="P6" s="46"/>
       <x:c r="Q6" s="46"/>
@@ -3152,24 +3152,25 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="E29" s="8" t="str">
-        <x:v>No iniciada</x:v>
+        <x:v>Completada</x:v>
       </x:c>
       <x:c r="F29" s="8" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="G29" s="49" t="n">
-        <x:v>46293</x:v>
+        <x:v>46235</x:v>
       </x:c>
       <x:c r="H29" s="49" t="n">
-        <x:v>46304</x:v>
+        <x:v>46235</x:v>
       </x:c>
       <x:c r="I29" s="11" t="n">
         <x:f t="shared" si="1">IF(OR(G29="",H29="",H29&lt;G29),"",H29-G29+1)</x:f>
-        <x:v>12</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J29" s="15"/>
-      <x:c r="K29" s="12" t="str">
+      <x:c r="K29" s="12" t="n">
         <x:f t="shared" si="4">IF(OR($G29="",$H29="",$H29&lt;$G29),"",IF(AND(K$9&lt;=$H29,K$9+6&gt;=$G29),1,""))</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L29" s="13" t="str">
         <x:f t="shared" si="4">IF(OR($G29="",$H29="",$H29&lt;$G29),"",IF(AND(L$9&lt;=$H29,L$9+6&gt;=$G29),1,""))</x:f>
@@ -3192,17 +3193,14 @@
       <x:c r="R29" s="13" t="str">
         <x:f t="shared" si="4">IF(OR($G29="",$H29="",$H29&lt;$G29),"",IF(AND(R$9&lt;=$H29,R$9+6&gt;=$G29),1,""))</x:f>
       </x:c>
-      <x:c r="S29" s="12" t="n">
+      <x:c r="S29" s="12" t="str">
         <x:f t="shared" si="4">IF(OR($G29="",$H29="",$H29&lt;$G29),"",IF(AND(S$9&lt;=$H29,S$9+6&gt;=$G29),1,""))</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="T29" s="13" t="n">
+      </x:c>
+      <x:c r="T29" s="13" t="str">
         <x:f t="shared" si="4">IF(OR($G29="",$H29="",$H29&lt;$G29),"",IF(AND(T$9&lt;=$H29,T$9+6&gt;=$G29),1,""))</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U29" s="12" t="n">
+      </x:c>
+      <x:c r="U29" s="12" t="str">
         <x:f t="shared" si="5">IF(OR($G29="",$H29="",$H29&lt;$G29),"",IF(AND(U$9&lt;=$H29,U$9+6&gt;=$G29),1,""))</x:f>
-        <x:v>1</x:v>
       </x:c>
       <x:c r="V29" s="13" t="str">
         <x:f t="shared" si="5">IF(OR($G29="",$H29="",$H29&lt;$G29),"",IF(AND(V$9&lt;=$H29,V$9+6&gt;=$G29),1,""))</x:f>
@@ -3243,24 +3241,25 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="E30" s="7" t="str">
-        <x:v>No iniciada</x:v>
+        <x:v>Completada</x:v>
       </x:c>
       <x:c r="F30" s="7" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="G30" s="48" t="n">
-        <x:v>46300</x:v>
+        <x:v>46235</x:v>
       </x:c>
       <x:c r="H30" s="48" t="n">
-        <x:v>46308</x:v>
+        <x:v>46235</x:v>
       </x:c>
       <x:c r="I30" s="11" t="n">
         <x:f t="shared" si="1">IF(OR(G30="",H30="",H30&lt;G30),"",H30-G30+1)</x:f>
-        <x:v>9</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J30" s="15"/>
-      <x:c r="K30" s="12" t="str">
+      <x:c r="K30" s="12" t="n">
         <x:f t="shared" ref="K30:T39" si="6">IF(OR($G30="",$H30="",$H30&lt;$G30),"",IF(AND(K$9&lt;=$H30,K$9+6&gt;=$G30),1,""))</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L30" s="13" t="str">
         <x:f t="shared" si="6">IF(OR($G30="",$H30="",$H30&lt;$G30),"",IF(AND(L$9&lt;=$H30,L$9+6&gt;=$G30),1,""))</x:f>
@@ -3286,13 +3285,11 @@
       <x:c r="S30" s="12" t="str">
         <x:f t="shared" si="6">IF(OR($G30="",$H30="",$H30&lt;$G30),"",IF(AND(S$9&lt;=$H30,S$9+6&gt;=$G30),1,""))</x:f>
       </x:c>
-      <x:c r="T30" s="13" t="n">
+      <x:c r="T30" s="13" t="str">
         <x:f t="shared" si="6">IF(OR($G30="",$H30="",$H30&lt;$G30),"",IF(AND(T$9&lt;=$H30,T$9+6&gt;=$G30),1,""))</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U30" s="12" t="n">
+      </x:c>
+      <x:c r="U30" s="12" t="str">
         <x:f t="shared" ref="U30:AD39" si="7">IF(OR($G30="",$H30="",$H30&lt;$G30),"",IF(AND(U$9&lt;=$H30,U$9+6&gt;=$G30),1,""))</x:f>
-        <x:v>1</x:v>
       </x:c>
       <x:c r="V30" s="13" t="str">
         <x:f t="shared" si="7">IF(OR($G30="",$H30="",$H30&lt;$G30),"",IF(AND(V$9&lt;=$H30,V$9+6&gt;=$G30),1,""))</x:f>
@@ -3330,27 +3327,28 @@
         <x:v>Preparar incorporación segura de dispositivos</x:v>
       </x:c>
       <x:c r="D31" s="59" t="str">
-        <x:v>Codex + Lucas</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="E31" s="8" t="str">
-        <x:v>No iniciada</x:v>
+        <x:v>Completada</x:v>
       </x:c>
       <x:c r="F31" s="8" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="G31" s="50" t="n">
-        <x:v>46302</x:v>
+        <x:v>46235</x:v>
       </x:c>
       <x:c r="H31" s="50" t="n">
-        <x:v>46311</x:v>
+        <x:v>46235</x:v>
       </x:c>
       <x:c r="I31" s="11" t="n">
         <x:f t="shared" si="1">IF(OR(G31="",H31="",H31&lt;G31),"",H31-G31+1)</x:f>
-        <x:v>10</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J31" s="15"/>
-      <x:c r="K31" s="12" t="str">
+      <x:c r="K31" s="12" t="n">
         <x:f t="shared" si="6">IF(OR($G31="",$H31="",$H31&lt;$G31),"",IF(AND(K$9&lt;=$H31,K$9+6&gt;=$G31),1,""))</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L31" s="13" t="str">
         <x:f t="shared" si="6">IF(OR($G31="",$H31="",$H31&lt;$G31),"",IF(AND(L$9&lt;=$H31,L$9+6&gt;=$G31),1,""))</x:f>
@@ -3379,13 +3377,11 @@
       <x:c r="T31" s="13" t="str">
         <x:f t="shared" si="6">IF(OR($G31="",$H31="",$H31&lt;$G31),"",IF(AND(T$9&lt;=$H31,T$9+6&gt;=$G31),1,""))</x:f>
       </x:c>
-      <x:c r="U31" s="12" t="n">
+      <x:c r="U31" s="12" t="str">
         <x:f t="shared" si="7">IF(OR($G31="",$H31="",$H31&lt;$G31),"",IF(AND(U$9&lt;=$H31,U$9+6&gt;=$G31),1,""))</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="V31" s="13" t="n">
+      </x:c>
+      <x:c r="V31" s="13" t="str">
         <x:f t="shared" si="7">IF(OR($G31="",$H31="",$H31&lt;$G31),"",IF(AND(V$9&lt;=$H31,V$9+6&gt;=$G31),1,""))</x:f>
-        <x:v>1</x:v>
       </x:c>
       <x:c r="W31" s="12" t="str">
         <x:f t="shared" si="7">IF(OR($G31="",$H31="",$H31&lt;$G31),"",IF(AND(W$9&lt;=$H31,W$9+6&gt;=$G31),1,""))</x:f>
@@ -3696,24 +3692,25 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="E35" s="8" t="str">
-        <x:v>No iniciada</x:v>
+        <x:v>Completada</x:v>
       </x:c>
       <x:c r="F35" s="8" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="G35" s="50" t="n">
-        <x:v>46328</x:v>
+        <x:v>46235</x:v>
       </x:c>
       <x:c r="H35" s="50" t="n">
-        <x:v>46336</x:v>
+        <x:v>46235</x:v>
       </x:c>
       <x:c r="I35" s="11" t="n">
         <x:f t="shared" si="1">IF(OR(G35="",H35="",H35&lt;G35),"",H35-G35+1)</x:f>
-        <x:v>9</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J35" s="15"/>
-      <x:c r="K35" s="12" t="str">
+      <x:c r="K35" s="12" t="n">
         <x:f t="shared" si="6">IF(OR($G35="",$H35="",$H35&lt;$G35),"",IF(AND(K$9&lt;=$H35,K$9+6&gt;=$G35),1,""))</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L35" s="13" t="str">
         <x:f t="shared" si="6">IF(OR($G35="",$H35="",$H35&lt;$G35),"",IF(AND(L$9&lt;=$H35,L$9+6&gt;=$G35),1,""))</x:f>
@@ -3751,13 +3748,11 @@
       <x:c r="W35" s="12" t="str">
         <x:f t="shared" si="7">IF(OR($G35="",$H35="",$H35&lt;$G35),"",IF(AND(W$9&lt;=$H35,W$9+6&gt;=$G35),1,""))</x:f>
       </x:c>
-      <x:c r="X35" s="13" t="n">
+      <x:c r="X35" s="13" t="str">
         <x:f t="shared" si="7">IF(OR($G35="",$H35="",$H35&lt;$G35),"",IF(AND(X$9&lt;=$H35,X$9+6&gt;=$G35),1,""))</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="Y35" s="12" t="n">
+      </x:c>
+      <x:c r="Y35" s="12" t="str">
         <x:f t="shared" si="7">IF(OR($G35="",$H35="",$H35&lt;$G35),"",IF(AND(Y$9&lt;=$H35,Y$9+6&gt;=$G35),1,""))</x:f>
-        <x:v>1</x:v>
       </x:c>
       <x:c r="Z35" s="13" t="str">
         <x:f t="shared" si="7">IF(OR($G35="",$H35="",$H35&lt;$G35),"",IF(AND(Z$9&lt;=$H35,Z$9+6&gt;=$G35),1,""))</x:f>
@@ -4172,180 +4167,180 @@
     </x:row>
     <x:row r="41" ht="24" customHeight="1">
       <x:c r="B41" s="60" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="C41" s="61" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="D41" s="61" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="E41" s="61" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="F41" s="61" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="G41" s="61" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="H41" s="61" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="I41" s="61" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="J41" s="61" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="K41" s="61" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="L41" s="61" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="M41" s="61" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="N41" s="61" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="O41" s="61" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="P41" s="61" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="Q41" s="61" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="R41" s="61" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="S41" s="61" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="T41" s="61" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="U41" s="61" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="V41" s="61" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="W41" s="61" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="X41" s="61" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="Y41" s="61" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="Z41" s="61" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="AA41" s="61" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="AB41" s="61" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="AC41" s="61" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="AD41" s="62" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="24" customHeight="1">
       <x:c r="B42" s="63" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="C42" s="64" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="D42" s="64" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="E42" s="64" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="F42" s="64" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="G42" s="64" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="H42" s="64" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="I42" s="64" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="J42" s="64" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="K42" s="64" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="L42" s="64" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="M42" s="64" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="N42" s="64" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="O42" s="64" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="P42" s="64" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="Q42" s="64" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="R42" s="64" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="S42" s="64" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="T42" s="64" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="U42" s="64" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="V42" s="64" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="W42" s="64" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="X42" s="64" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="Y42" s="64" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="Z42" s="64" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="AA42" s="64" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="AB42" s="64" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="AC42" s="64" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="AD42" s="65" t="str">
-        <x:v>Reglas del plan: el Excel ERP no se modifica; las exportaciones enriquecidas son propias; cada cambio sensible debe auditarse; la cámara móvil requiere HTTPS interno; ninguna regularización puede duplicar estudiantes ni perder historial.</x:v>
+        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
mod: actualizar tracker con auditoria y cierre tecnico
</commit_message>
<xml_diff>
--- a/outputs/ldsm-identidad-20260729/Tracker_Implementacion_Identidad_y_Registro_Movil_LDSM.xlsx
+++ b/outputs/ldsm-identidad-20260729/Tracker_Implementacion_Identidad_y_Registro_Movil_LDSM.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Plan" sheetId="1" r:id="Rd915ee891ba54079"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Plan" sheetId="1" r:id="R5a80e6a2401241a4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1198,7 +1198,7 @@
       <x:c r="N6" s="44"/>
       <x:c r="O6" s="45" t="n">
         <x:f>COUNTIF($E$10:$E$39,"Completada")</x:f>
-        <x:v>23</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="P6" s="46"/>
       <x:c r="Q6" s="46"/>
@@ -3413,10 +3413,10 @@
         <x:v>HTTPS interno</x:v>
       </x:c>
       <x:c r="C32" s="56" t="str">
-        <x:v>Probar cámara en Android y escritorios</x:v>
+        <x:v>Instalar certificado y probar cámara en dispositivos del colegio</x:v>
       </x:c>
       <x:c r="D32" s="58" t="str">
-        <x:v>Lucas</x:v>
+        <x:v>Lucas + LDSM</x:v>
       </x:c>
       <x:c r="E32" s="7" t="str">
         <x:v>No iniciada</x:v>
@@ -3510,24 +3510,25 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="E33" s="8" t="str">
-        <x:v>No iniciada</x:v>
+        <x:v>Completada</x:v>
       </x:c>
       <x:c r="F33" s="8" t="str">
         <x:v>P2</x:v>
       </x:c>
       <x:c r="G33" s="50" t="n">
-        <x:v>46314</x:v>
+        <x:v>46235</x:v>
       </x:c>
       <x:c r="H33" s="50" t="n">
-        <x:v>46325</x:v>
+        <x:v>46235</x:v>
       </x:c>
       <x:c r="I33" s="11" t="n">
         <x:f t="shared" si="1">IF(OR(G33="",H33="",H33&lt;G33),"",H33-G33+1)</x:f>
-        <x:v>12</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J33" s="15"/>
-      <x:c r="K33" s="12" t="str">
+      <x:c r="K33" s="12" t="n">
         <x:f t="shared" si="6">IF(OR($G33="",$H33="",$H33&lt;$G33),"",IF(AND(K$9&lt;=$H33,K$9+6&gt;=$G33),1,""))</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L33" s="13" t="str">
         <x:f t="shared" si="6">IF(OR($G33="",$H33="",$H33&lt;$G33),"",IF(AND(L$9&lt;=$H33,L$9+6&gt;=$G33),1,""))</x:f>
@@ -3559,17 +3560,14 @@
       <x:c r="U33" s="12" t="str">
         <x:f t="shared" si="7">IF(OR($G33="",$H33="",$H33&lt;$G33),"",IF(AND(U$9&lt;=$H33,U$9+6&gt;=$G33),1,""))</x:f>
       </x:c>
-      <x:c r="V33" s="13" t="n">
+      <x:c r="V33" s="13" t="str">
         <x:f t="shared" si="7">IF(OR($G33="",$H33="",$H33&lt;$G33),"",IF(AND(V$9&lt;=$H33,V$9+6&gt;=$G33),1,""))</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="W33" s="12" t="n">
+      </x:c>
+      <x:c r="W33" s="12" t="str">
         <x:f t="shared" si="7">IF(OR($G33="",$H33="",$H33&lt;$G33),"",IF(AND(W$9&lt;=$H33,W$9+6&gt;=$G33),1,""))</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="X33" s="13" t="n">
+      </x:c>
+      <x:c r="X33" s="13" t="str">
         <x:f t="shared" si="7">IF(OR($G33="",$H33="",$H33&lt;$G33),"",IF(AND(X$9&lt;=$H33,X$9+6&gt;=$G33),1,""))</x:f>
-        <x:v>1</x:v>
       </x:c>
       <x:c r="Y33" s="12" t="str">
         <x:f t="shared" si="7">IF(OR($G33="",$H33="",$H33&lt;$G33),"",IF(AND(Y$9&lt;=$H33,Y$9+6&gt;=$G33),1,""))</x:f>
@@ -3601,24 +3599,25 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="E34" s="7" t="str">
-        <x:v>No iniciada</x:v>
+        <x:v>Completada</x:v>
       </x:c>
       <x:c r="F34" s="7" t="str">
         <x:v>P2</x:v>
       </x:c>
       <x:c r="G34" s="51" t="n">
-        <x:v>46321</x:v>
+        <x:v>46235</x:v>
       </x:c>
       <x:c r="H34" s="51" t="n">
-        <x:v>46332</x:v>
+        <x:v>46235</x:v>
       </x:c>
       <x:c r="I34" s="11" t="n">
         <x:f t="shared" si="1">IF(OR(G34="",H34="",H34&lt;G34),"",H34-G34+1)</x:f>
-        <x:v>12</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J34" s="15"/>
-      <x:c r="K34" s="12" t="str">
+      <x:c r="K34" s="12" t="n">
         <x:f t="shared" si="6">IF(OR($G34="",$H34="",$H34&lt;$G34),"",IF(AND(K$9&lt;=$H34,K$9+6&gt;=$G34),1,""))</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L34" s="13" t="str">
         <x:f t="shared" si="6">IF(OR($G34="",$H34="",$H34&lt;$G34),"",IF(AND(L$9&lt;=$H34,L$9+6&gt;=$G34),1,""))</x:f>
@@ -3653,17 +3652,14 @@
       <x:c r="V34" s="13" t="str">
         <x:f t="shared" si="7">IF(OR($G34="",$H34="",$H34&lt;$G34),"",IF(AND(V$9&lt;=$H34,V$9+6&gt;=$G34),1,""))</x:f>
       </x:c>
-      <x:c r="W34" s="12" t="n">
+      <x:c r="W34" s="12" t="str">
         <x:f t="shared" si="7">IF(OR($G34="",$H34="",$H34&lt;$G34),"",IF(AND(W$9&lt;=$H34,W$9+6&gt;=$G34),1,""))</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="X34" s="13" t="n">
+      </x:c>
+      <x:c r="X34" s="13" t="str">
         <x:f t="shared" si="7">IF(OR($G34="",$H34="",$H34&lt;$G34),"",IF(AND(X$9&lt;=$H34,X$9+6&gt;=$G34),1,""))</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="Y34" s="12" t="n">
+      </x:c>
+      <x:c r="Y34" s="12" t="str">
         <x:f t="shared" si="7">IF(OR($G34="",$H34="",$H34&lt;$G34),"",IF(AND(Y$9&lt;=$H34,Y$9+6&gt;=$G34),1,""))</x:f>
-        <x:v>1</x:v>
       </x:c>
       <x:c r="Z34" s="13" t="str">
         <x:f t="shared" si="7">IF(OR($G34="",$H34="",$H34&lt;$G34),"",IF(AND(Z$9&lt;=$H34,Z$9+6&gt;=$G34),1,""))</x:f>
@@ -3781,24 +3777,25 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="E36" s="7" t="str">
-        <x:v>No iniciada</x:v>
+        <x:v>Completada</x:v>
       </x:c>
       <x:c r="F36" s="7" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="G36" s="51" t="n">
-        <x:v>46331</x:v>
+        <x:v>46235</x:v>
       </x:c>
       <x:c r="H36" s="51" t="n">
-        <x:v>46344</x:v>
+        <x:v>46235</x:v>
       </x:c>
       <x:c r="I36" s="11" t="n">
         <x:f t="shared" si="1">IF(OR(G36="",H36="",H36&lt;G36),"",H36-G36+1)</x:f>
-        <x:v>14</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J36" s="15"/>
-      <x:c r="K36" s="12" t="str">
+      <x:c r="K36" s="12" t="n">
         <x:f t="shared" si="6">IF(OR($G36="",$H36="",$H36&lt;$G36),"",IF(AND(K$9&lt;=$H36,K$9+6&gt;=$G36),1,""))</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L36" s="13" t="str">
         <x:f t="shared" si="6">IF(OR($G36="",$H36="",$H36&lt;$G36),"",IF(AND(L$9&lt;=$H36,L$9+6&gt;=$G36),1,""))</x:f>
@@ -3839,17 +3836,14 @@
       <x:c r="X36" s="13" t="str">
         <x:f t="shared" si="7">IF(OR($G36="",$H36="",$H36&lt;$G36),"",IF(AND(X$9&lt;=$H36,X$9+6&gt;=$G36),1,""))</x:f>
       </x:c>
-      <x:c r="Y36" s="12" t="n">
+      <x:c r="Y36" s="12" t="str">
         <x:f t="shared" si="7">IF(OR($G36="",$H36="",$H36&lt;$G36),"",IF(AND(Y$9&lt;=$H36,Y$9+6&gt;=$G36),1,""))</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="Z36" s="13" t="n">
+      </x:c>
+      <x:c r="Z36" s="13" t="str">
         <x:f t="shared" si="7">IF(OR($G36="",$H36="",$H36&lt;$G36),"",IF(AND(Z$9&lt;=$H36,Z$9+6&gt;=$G36),1,""))</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AA36" s="12" t="n">
+      </x:c>
+      <x:c r="AA36" s="12" t="str">
         <x:f t="shared" si="7">IF(OR($G36="",$H36="",$H36&lt;$G36),"",IF(AND(AA$9&lt;=$H36,AA$9+6&gt;=$G36),1,""))</x:f>
-        <x:v>1</x:v>
       </x:c>
       <x:c r="AB36" s="13" t="str">
         <x:f t="shared" si="7">IF(OR($G36="",$H36="",$H36&lt;$G36),"",IF(AND(AB$9&lt;=$H36,AB$9+6&gt;=$G36),1,""))</x:f>
@@ -3869,27 +3863,28 @@
         <x:v>E2E móvil, permisos y datos sensibles</x:v>
       </x:c>
       <x:c r="D37" s="59" t="str">
-        <x:v>Codex + Lucas</x:v>
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="E37" s="8" t="str">
-        <x:v>No iniciada</x:v>
+        <x:v>Completada</x:v>
       </x:c>
       <x:c r="F37" s="8" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="G37" s="50" t="n">
-        <x:v>46338</x:v>
+        <x:v>46235</x:v>
       </x:c>
       <x:c r="H37" s="50" t="n">
-        <x:v>46351</x:v>
+        <x:v>46235</x:v>
       </x:c>
       <x:c r="I37" s="11" t="n">
         <x:f t="shared" si="1">IF(OR(G37="",H37="",H37&lt;G37),"",H37-G37+1)</x:f>
-        <x:v>14</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J37" s="15"/>
-      <x:c r="K37" s="12" t="str">
+      <x:c r="K37" s="12" t="n">
         <x:f t="shared" si="6">IF(OR($G37="",$H37="",$H37&lt;$G37),"",IF(AND(K$9&lt;=$H37,K$9+6&gt;=$G37),1,""))</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L37" s="13" t="str">
         <x:f t="shared" si="6">IF(OR($G37="",$H37="",$H37&lt;$G37),"",IF(AND(L$9&lt;=$H37,L$9+6&gt;=$G37),1,""))</x:f>
@@ -3933,17 +3928,14 @@
       <x:c r="Y37" s="12" t="str">
         <x:f t="shared" si="7">IF(OR($G37="",$H37="",$H37&lt;$G37),"",IF(AND(Y$9&lt;=$H37,Y$9+6&gt;=$G37),1,""))</x:f>
       </x:c>
-      <x:c r="Z37" s="13" t="n">
+      <x:c r="Z37" s="13" t="str">
         <x:f t="shared" si="7">IF(OR($G37="",$H37="",$H37&lt;$G37),"",IF(AND(Z$9&lt;=$H37,Z$9+6&gt;=$G37),1,""))</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AA37" s="12" t="n">
+      </x:c>
+      <x:c r="AA37" s="12" t="str">
         <x:f t="shared" si="7">IF(OR($G37="",$H37="",$H37&lt;$G37),"",IF(AND(AA$9&lt;=$H37,AA$9+6&gt;=$G37),1,""))</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AB37" s="13" t="n">
+      </x:c>
+      <x:c r="AB37" s="13" t="str">
         <x:f t="shared" si="7">IF(OR($G37="",$H37="",$H37&lt;$G37),"",IF(AND(AB$9&lt;=$H37,AB$9+6&gt;=$G37),1,""))</x:f>
-        <x:v>1</x:v>
       </x:c>
       <x:c r="AC37" s="12" t="str">
         <x:f t="shared" si="7">IF(OR($G37="",$H37="",$H37&lt;$G37),"",IF(AND(AC$9&lt;=$H37,AC$9+6&gt;=$G37),1,""))</x:f>
@@ -3957,30 +3949,31 @@
         <x:v>QA</x:v>
       </x:c>
       <x:c r="C38" s="56" t="str">
-        <x:v>Recuperación, rendimiento y accesibilidad</x:v>
+        <x:v>Recuperación, rendimiento, accesibilidad y manuales</x:v>
       </x:c>
       <x:c r="D38" s="58" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="E38" s="7" t="str">
-        <x:v>No iniciada</x:v>
+        <x:v>Completada</x:v>
       </x:c>
       <x:c r="F38" s="7" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="G38" s="51" t="n">
-        <x:v>46346</x:v>
+        <x:v>46235</x:v>
       </x:c>
       <x:c r="H38" s="51" t="n">
-        <x:v>46360</x:v>
+        <x:v>46235</x:v>
       </x:c>
       <x:c r="I38" s="11" t="n">
         <x:f t="shared" si="1">IF(OR(G38="",H38="",H38&lt;G38),"",H38-G38+1)</x:f>
-        <x:v>15</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J38" s="15"/>
-      <x:c r="K38" s="12" t="str">
+      <x:c r="K38" s="12" t="n">
         <x:f t="shared" si="6">IF(OR($G38="",$H38="",$H38&lt;$G38),"",IF(AND(K$9&lt;=$H38,K$9+6&gt;=$G38),1,""))</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L38" s="13" t="str">
         <x:f t="shared" si="6">IF(OR($G38="",$H38="",$H38&lt;$G38),"",IF(AND(L$9&lt;=$H38,L$9+6&gt;=$G38),1,""))</x:f>
@@ -4027,17 +4020,14 @@
       <x:c r="Z38" s="13" t="str">
         <x:f t="shared" si="7">IF(OR($G38="",$H38="",$H38&lt;$G38),"",IF(AND(Z$9&lt;=$H38,Z$9+6&gt;=$G38),1,""))</x:f>
       </x:c>
-      <x:c r="AA38" s="12" t="n">
+      <x:c r="AA38" s="12" t="str">
         <x:f t="shared" si="7">IF(OR($G38="",$H38="",$H38&lt;$G38),"",IF(AND(AA$9&lt;=$H38,AA$9+6&gt;=$G38),1,""))</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AB38" s="13" t="n">
+      </x:c>
+      <x:c r="AB38" s="13" t="str">
         <x:f t="shared" si="7">IF(OR($G38="",$H38="",$H38&lt;$G38),"",IF(AND(AB$9&lt;=$H38,AB$9+6&gt;=$G38),1,""))</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AC38" s="12" t="n">
+      </x:c>
+      <x:c r="AC38" s="12" t="str">
         <x:f t="shared" si="7">IF(OR($G38="",$H38="",$H38&lt;$G38),"",IF(AND(AC$9&lt;=$H38,AC$9+6&gt;=$G38),1,""))</x:f>
-        <x:v>1</x:v>
       </x:c>
       <x:c r="AD38" s="13" t="str">
         <x:f t="shared" si="7">IF(OR($G38="",$H38="",$H38&lt;$G38),"",IF(AND(AD$9&lt;=$H38,AD$9+6&gt;=$G38),1,""))</x:f>
@@ -4048,7 +4038,7 @@
         <x:v>Aceptación</x:v>
       </x:c>
       <x:c r="C39" s="57" t="str">
-        <x:v>Auditoría final, manuales y aprobación escolar</x:v>
+        <x:v>Prueba física, capacitación y aprobación escolar</x:v>
       </x:c>
       <x:c r="D39" s="59" t="str">
         <x:v>Lucas + LDSM</x:v>
@@ -4167,180 +4157,180 @@
     </x:row>
     <x:row r="41" ht="24" customHeight="1">
       <x:c r="B41" s="60" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="C41" s="61" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="D41" s="61" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="E41" s="61" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="F41" s="61" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="G41" s="61" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="H41" s="61" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="I41" s="61" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="J41" s="61" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="K41" s="61" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="L41" s="61" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="M41" s="61" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="N41" s="61" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="O41" s="61" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="P41" s="61" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="Q41" s="61" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="R41" s="61" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="S41" s="61" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="T41" s="61" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="U41" s="61" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="V41" s="61" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="W41" s="61" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="X41" s="61" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="Y41" s="61" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="Z41" s="61" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="AA41" s="61" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="AB41" s="61" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="AC41" s="61" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="AD41" s="62" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="24" customHeight="1">
       <x:c r="B42" s="63" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="C42" s="64" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="D42" s="64" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="E42" s="64" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="F42" s="64" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="G42" s="64" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="H42" s="64" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="I42" s="64" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="J42" s="64" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="K42" s="64" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="L42" s="64" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="M42" s="64" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="N42" s="64" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="O42" s="64" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="P42" s="64" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="Q42" s="64" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="R42" s="64" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="S42" s="64" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="T42" s="64" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="U42" s="64" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="V42" s="64" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="W42" s="64" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="X42" s="64" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="Y42" s="64" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="Z42" s="64" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="AA42" s="64" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="AB42" s="64" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="AC42" s="64" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
       <x:c r="AD42" s="65" t="str">
-        <x:v>Estado al 1 ago 2026: cámara web, fallback manual, antiduplicado, permisos por método y preparación HTTPS completados; 102 pruebas backend y 11 frontend aprobadas. Pendiente físico: confiar el certificado y probar cámara en Android/escritorios del colegio. El Excel ERP no se modifica.</x:v>
+        <x:v>Estado al 1 ago 2026: 28 de 30 tareas completadas. Aprobadas 103 pruebas backend, 14 frontend y 9 E2E; ERP oficial 392 preparadas y 0 rechazadas; restauración aislada, accesibilidad, rendimiento y auditorías de dependencias aprobadas. Pendiente físico: certificado, cámara, capacitación y aceptación escolar. El Excel ERP no se modifica.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>